<commit_message>
DatDM7.FPT: Add the NCAP_Scenario folder and complete run the CPNA_AEB
</commit_message>
<xml_diff>
--- a/specifications/Test Scenarios.xlsx
+++ b/specifications/Test Scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OpenScenario\test_assets\requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="648" documentId="13_ncr:1_{F5A69BD8-62CC-4032-9E11-682A20827548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0ABCECC1-B3C3-420F-9F89-E47C7D997B59}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A7095C2B-65DA-42E9-B40B-AD56B40CBB93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0. SUM" sheetId="3" r:id="rId1"/>
@@ -28,6 +28,9 @@
     <sheet name="10. RCTA" sheetId="12" r:id="rId13"/>
     <sheet name="11. IA" sheetId="13" r:id="rId14"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'16. FAEB'!$B$2:$R$2</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -67,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="885" uniqueCount="429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="945" uniqueCount="445">
   <si>
     <t>Feature list</t>
   </si>
@@ -993,13 +996,17 @@
     <t>LKA_SCS_001</t>
   </si>
   <si>
-    <t>LKA_REQ_001/2/3/4</t>
+    <t>LKA_REQ_001
+LKA_REQ_002
+LKA_REQ_003
+LKA_REQ_004</t>
   </si>
   <si>
     <t>LKA intervention in working speed</t>
   </si>
   <si>
-    <t>LKA is enable</t>
+    <t>LKA is enable
+Road is straight</t>
   </si>
   <si>
     <r>
@@ -1026,7 +1033,236 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos"/>
       </rPr>
-      <t xml:space="preserve">2. EV run in a </t>
+      <t xml:space="preserve">2. Driver intervenes in to steering wheel to steer slightly EV to the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t>left</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t>, then release steering wheel</t>
+    </r>
+  </si>
+  <si>
+    <t>LKA active to pull EV back to ego lane</t>
+  </si>
+  <si>
+    <t>lka_csc_001</t>
+  </si>
+  <si>
+    <t>[50,100, 150]</t>
+  </si>
+  <si>
+    <t>[clear, rain, fog]</t>
+  </si>
+  <si>
+    <t>[White, Yellow]</t>
+  </si>
+  <si>
+    <t>[Solid, Dash]</t>
+  </si>
+  <si>
+    <t>LKA_SCS_002</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t xml:space="preserve">1. EV run on </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t xml:space="preserve">straight road
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t xml:space="preserve">2. Driver intervenes in to steering wheel to steer slightly EV to the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t>right</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t>, then release steering wheel</t>
+    </r>
+  </si>
+  <si>
+    <t>lka_csc_002</t>
+  </si>
+  <si>
+    <t>LKA_SCS_003</t>
+  </si>
+  <si>
+    <t>LKA is enable
+Road is curved</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t xml:space="preserve">1. EV run on a </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t xml:space="preserve">curve
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t xml:space="preserve">2. Driver intervenes in to steering wheel to steer slightly EV to the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t>left</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t>, then release steering wheel</t>
+    </r>
+  </si>
+  <si>
+    <t>lka_csc_003</t>
+  </si>
+  <si>
+    <t>[50, 75, 100]</t>
+  </si>
+  <si>
+    <t>LKA_SCS_004</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t xml:space="preserve">1. EV run on a </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t xml:space="preserve">curve
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t xml:space="preserve">2. Driver intervenes in to steering wheel to steer slightly EV to the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t>right</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t>, then release steering wheel</t>
+    </r>
+  </si>
+  <si>
+    <t>lka_csc_004</t>
+  </si>
+  <si>
+    <t>LKA_SCS_005</t>
+  </si>
+  <si>
+    <t>LKA is enable</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t xml:space="preserve">1. EV run on </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t xml:space="preserve">straight road
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t xml:space="preserve">2. EV run into a </t>
     </r>
     <r>
       <rPr>
@@ -1039,25 +1275,10 @@
     </r>
   </si>
   <si>
-    <t>LKA active to pull EV back to ego lane</t>
-  </si>
-  <si>
-    <t>lka_csc_001</t>
-  </si>
-  <si>
-    <t>[50,100, 150]</t>
-  </si>
-  <si>
-    <t>[clear, rain, fog]</t>
-  </si>
-  <si>
-    <t>[White, Yellow]</t>
-  </si>
-  <si>
-    <t>[Solid, Dash]</t>
-  </si>
-  <si>
-    <t>LKA_SCS_002</t>
+    <t>lka_csc_005</t>
+  </si>
+  <si>
+    <t>LKA_SCS_006</t>
   </si>
   <si>
     <r>
@@ -1084,7 +1305,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos"/>
       </rPr>
-      <t xml:space="preserve">2. EV run in to </t>
+      <t xml:space="preserve">2. EV run into </t>
     </r>
     <r>
       <rPr>
@@ -1097,10 +1318,10 @@
     </r>
   </si>
   <si>
-    <t>lka_csc_002</t>
-  </si>
-  <si>
-    <t>LKA_SCS_003</t>
+    <t>lka_csc_006</t>
+  </si>
+  <si>
+    <t>LKA_SCS_007</t>
   </si>
   <si>
     <t>LKA intervention in working speed boundary</t>
@@ -1110,13 +1331,13 @@
 2. EV run in a slight curve</t>
   </si>
   <si>
-    <t>lka_csc_003</t>
+    <t>lka_csc_007</t>
   </si>
   <si>
     <t>[45,155]</t>
   </si>
   <si>
-    <t>LKA_SCS_004</t>
+    <t>LKA_SCS_008</t>
   </si>
   <si>
     <t>LKA intervention in lane width boundary, driver slight steers to the left</t>
@@ -1127,13 +1348,13 @@
 3. Put steering wheel intervene signal into EV in 1 second: slightly steer to the left</t>
   </si>
   <si>
-    <t>lka_csc_004</t>
+    <t>lka_csc_008</t>
   </si>
   <si>
     <t>[2.5; 5.5]</t>
   </si>
   <si>
-    <t>LKA_SCS_005</t>
+    <t>LKA_SCS_009</t>
   </si>
   <si>
     <t>LKA intervention in lane width boundary, driver slight steers to the right</t>
@@ -1144,10 +1365,10 @@
 3. Put steering wheel intervene signal into EV in 1 second: slight steer to the right</t>
   </si>
   <si>
-    <t>lka_csc_005</t>
-  </si>
-  <si>
-    <t>LKA_SCS_006</t>
+    <t>lka_csc_009</t>
+  </si>
+  <si>
+    <t>LKA_SCS_010</t>
   </si>
   <si>
     <t>LKA intervention in working slope boundary, driver slight steers to the left</t>
@@ -1158,10 +1379,10 @@
 3. Put steering wheel intervene signal into EV in 1 second: slight steer to the left</t>
   </si>
   <si>
-    <t>lka_csc_006</t>
-  </si>
-  <si>
-    <t>LKA_SCS_007</t>
+    <t>lka_csc_010</t>
+  </si>
+  <si>
+    <t>LKA_SCS_011</t>
   </si>
   <si>
     <t>LKA intervention in working slope boundary, driver slight steers to the right</t>
@@ -1172,10 +1393,10 @@
 3. Put steering wheel intervene signal into EV in 1 second: slight steer to the right</t>
   </si>
   <si>
-    <t>lka_csc_007</t>
-  </si>
-  <si>
-    <t>LKA_SCS_008</t>
+    <t>lka_csc_011</t>
+  </si>
+  <si>
+    <t>LKA_SCS_012</t>
   </si>
   <si>
     <t>LKA intervention in curve radius boundary</t>
@@ -1185,14 +1406,14 @@
 2. EV run in a curve which radius is in boundary value (select from Simulation Maps)</t>
   </si>
   <si>
-    <t>lka_csc_008</t>
+    <t>lka_csc_012</t>
   </si>
   <si>
     <t>Target_speed (post-reduce)
 (kph)</t>
   </si>
   <si>
-    <t>FAEB_CSC_001</t>
+    <t>AEB_CSC_001</t>
   </si>
   <si>
     <t>FAEB_REQ_001
@@ -1215,10 +1436,10 @@
     <t>EV brakes to stop</t>
   </si>
   <si>
-    <t>FAEB_csc_001</t>
-  </si>
-  <si>
-    <t>FAEB_par_001</t>
+    <t>aeb_csc_001</t>
+  </si>
+  <si>
+    <t>aeb_par_001</t>
   </si>
   <si>
     <t>[10, 65, 120]</t>
@@ -1233,16 +1454,16 @@
     <t>[day, night]</t>
   </si>
   <si>
-    <t>FAEB_CSC_002</t>
+    <t>AEB_CSC_002</t>
   </si>
   <si>
     <t>FAEB active with moving vehicle, boundary EV speed</t>
   </si>
   <si>
-    <t>FAEB_csc_002</t>
-  </si>
-  <si>
-    <t>FAEB_par_002</t>
+    <t>aeb_csc_002</t>
+  </si>
+  <si>
+    <t>aeb_par_002</t>
   </si>
   <si>
     <t>[5, 130]</t>
@@ -1251,7 +1472,7 @@
     <t>[1, 26]</t>
   </si>
   <si>
-    <t>FAEB_CSC_003</t>
+    <t>AEB_CSC_003</t>
   </si>
   <si>
     <t>FAEB_REQ_003
@@ -1267,31 +1488,31 @@
     <t>TV is stoping, EV moves to approach TV</t>
   </si>
   <si>
-    <t>FAEB_csc_003</t>
-  </si>
-  <si>
-    <t>FAEB_par_003</t>
+    <t>aeb_csc_003</t>
+  </si>
+  <si>
+    <t>aeb_par_003</t>
   </si>
   <si>
     <t>[10, 40, 75]</t>
   </si>
   <si>
-    <t>FAEB_CSC_004</t>
+    <t>AEB_CSC_004</t>
   </si>
   <si>
     <t>FAEB active with stop vehicle, boundary EV speed</t>
   </si>
   <si>
-    <t>FAEB_csc_004</t>
-  </si>
-  <si>
-    <t>FAEB_par_004</t>
+    <t>aeb_csc_004</t>
+  </si>
+  <si>
+    <t>aeb_par_004</t>
   </si>
   <si>
     <t>[5, 80]</t>
   </si>
   <si>
-    <t>FAEB_CSC_005</t>
+    <t>AEB_CSC_005</t>
   </si>
   <si>
     <t>FAEB_REQ_003
@@ -1308,37 +1529,40 @@
 VRU is available infront of EV</t>
   </si>
   <si>
+    <t>VRU slowdown suddenly until EV-VRU distance reach TTC</t>
+  </si>
+  <si>
+    <t>aeb_csc_005</t>
+  </si>
+  <si>
+    <t>aeb_par_005</t>
+  </si>
+  <si>
+    <t>[2, 8, 15]</t>
+  </si>
+  <si>
+    <t>[bike, adult, child]</t>
+  </si>
+  <si>
+    <t>AEB_CSC_006</t>
+  </si>
+  <si>
+    <t>FAEB active with moving VRU, boundary EV speed</t>
+  </si>
+  <si>
     <t>VRU slowdown suddenly until EV-TV distance reach TTC</t>
   </si>
   <si>
-    <t>FAEB_csc_005</t>
-  </si>
-  <si>
-    <t>FAEB_par_005</t>
-  </si>
-  <si>
-    <t>[2, 8, 15]</t>
-  </si>
-  <si>
-    <t>[bike, adult, child]</t>
-  </si>
-  <si>
-    <t>FAEB_CSC_006</t>
-  </si>
-  <si>
-    <t>FAEB active with moving VRU, boundary EV speed</t>
-  </si>
-  <si>
-    <t>FAEB_csc_006</t>
-  </si>
-  <si>
-    <t>FAEB_par_006</t>
+    <t>aeb_csc_006</t>
+  </si>
+  <si>
+    <t>aeb_par_006</t>
   </si>
   <si>
     <t>[1, 16]</t>
   </si>
   <si>
-    <t>FAEB_CSC_007</t>
+    <t>AEB_CSC_007</t>
   </si>
   <si>
     <t>FAEB_REQ_004
@@ -1354,31 +1578,31 @@
     <t>VRU is static, EV moves to approach VRU</t>
   </si>
   <si>
-    <t>FAEB_csc_007</t>
-  </si>
-  <si>
-    <t>FAEB_par_007</t>
+    <t>aeb_csc_007</t>
+  </si>
+  <si>
+    <t>aeb_par_007</t>
   </si>
   <si>
     <t>[10, 20, 55]</t>
   </si>
   <si>
-    <t>FAEB_CSC_008</t>
+    <t>AEB_CSC_008</t>
   </si>
   <si>
     <t>FAEB active with atation VRU, boundary EV speed</t>
   </si>
   <si>
-    <t>FAEB_csc_008</t>
-  </si>
-  <si>
-    <t>FAEB_par_008</t>
+    <t>aeb_csc_008</t>
+  </si>
+  <si>
+    <t>aeb_par_008</t>
   </si>
   <si>
     <t>[5, 60]</t>
   </si>
   <si>
-    <t>FAEB_CSC_009</t>
+    <t>AEB_CSC_009</t>
   </si>
   <si>
     <t>FAEB_REQ_005
@@ -1399,28 +1623,28 @@
 EV moves to approach VRU</t>
   </si>
   <si>
-    <t>FAEB_csc_009</t>
-  </si>
-  <si>
-    <t>FAEB_par_009</t>
+    <t>aeb_csc_009</t>
+  </si>
+  <si>
+    <t>aeb_par_009</t>
   </si>
   <si>
     <t>[1,5]</t>
   </si>
   <si>
-    <t>FAEB_CSC_010</t>
+    <t>AEB_CSC_010</t>
   </si>
   <si>
     <t>FAEB active with crossing VRU, boundary EV speed</t>
   </si>
   <si>
-    <t>FAEB_csc_010</t>
-  </si>
-  <si>
-    <t>FAEB_par_010</t>
-  </si>
-  <si>
-    <t>FAEB_CSC_011</t>
+    <t>aeb_csc_010</t>
+  </si>
+  <si>
+    <t>aeb_par_010</t>
+  </si>
+  <si>
+    <t>AEB_CSC_011</t>
   </si>
   <si>
     <t>FAEB_REQ_019</t>
@@ -1440,28 +1664,28 @@
     <t>EV does not active FAEB</t>
   </si>
   <si>
-    <t>FAEB_csc_011</t>
-  </si>
-  <si>
-    <t>FAEB_par_011</t>
-  </si>
-  <si>
-    <t>FAEB_CSC_012</t>
-  </si>
-  <si>
-    <t>FAEB_csc_012</t>
-  </si>
-  <si>
-    <t>FAEB_par_012</t>
-  </si>
-  <si>
-    <t>FAEB_CSC_013</t>
-  </si>
-  <si>
-    <t>FAEB_csc_013</t>
-  </si>
-  <si>
-    <t>FAEB_par_013</t>
+    <t>aeb_csc_011</t>
+  </si>
+  <si>
+    <t>aeb_par_011</t>
+  </si>
+  <si>
+    <t>AEB_CSC_012</t>
+  </si>
+  <si>
+    <t>aeb_csc_012</t>
+  </si>
+  <si>
+    <t>aeb_par_012</t>
+  </si>
+  <si>
+    <t>AEB_CSC_013</t>
+  </si>
+  <si>
+    <t>aeb_csc_013</t>
+  </si>
+  <si>
+    <t>aeb_par_013</t>
   </si>
 </sst>
 </file>
@@ -4323,12 +4547,13 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="A2:S10"/>
+  <dimension ref="A2:S14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.42578125" customWidth="1"/>
     <col min="2" max="2" width="14.28515625" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" customWidth="1"/>
+    <col min="3" max="3" width="16.5703125" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="21" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
     <col min="7" max="7" width="42.7109375" customWidth="1"/>
@@ -4380,13 +4605,13 @@
         <v>302</v>
       </c>
       <c r="O2" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="P2" s="15" t="s">
         <v>303</v>
       </c>
-      <c r="P2" s="15" t="s">
+      <c r="Q2" s="15" t="s">
         <v>304</v>
-      </c>
-      <c r="Q2" s="15" t="s">
-        <v>62</v>
       </c>
       <c r="R2" s="15" t="s">
         <v>305</v>
@@ -4395,7 +4620,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="57.75">
+    <row r="3" spans="1:19" ht="66" customHeight="1">
       <c r="A3" s="19"/>
       <c r="B3" s="17" t="s">
         <v>306</v>
@@ -4448,7 +4673,7 @@
       <c r="R3" s="17"/>
       <c r="S3" s="17"/>
     </row>
-    <row r="4" spans="1:19" ht="57.75">
+    <row r="4" spans="1:19" ht="66" customHeight="1">
       <c r="A4" s="19"/>
       <c r="B4" s="17" t="s">
         <v>317</v>
@@ -4501,7 +4726,7 @@
       <c r="R4" s="17"/>
       <c r="S4" s="17"/>
     </row>
-    <row r="5" spans="1:19" ht="43.5">
+    <row r="5" spans="1:19" ht="66" customHeight="1">
       <c r="A5" s="19"/>
       <c r="B5" s="17" t="s">
         <v>320</v>
@@ -4510,15 +4735,15 @@
         <v>307</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="E5" s="17" t="s">
+        <v>308</v>
+      </c>
+      <c r="F5" s="17" t="s">
         <v>321</v>
       </c>
-      <c r="F5" s="17" t="s">
-        <v>309</v>
-      </c>
-      <c r="G5" s="17" t="s">
+      <c r="G5" s="21" t="s">
         <v>322</v>
       </c>
       <c r="H5" s="17" t="s">
@@ -4542,8 +4767,8 @@
       <c r="N5" s="17" t="s">
         <v>316</v>
       </c>
-      <c r="O5" s="17" t="s">
-        <v>74</v>
+      <c r="O5" s="17">
+        <v>300</v>
       </c>
       <c r="P5" s="17" t="s">
         <v>74</v>
@@ -4554,7 +4779,7 @@
       <c r="R5" s="17"/>
       <c r="S5" s="17"/>
     </row>
-    <row r="6" spans="1:19" ht="87">
+    <row r="6" spans="1:19" ht="66" customHeight="1">
       <c r="A6" s="19"/>
       <c r="B6" s="17" t="s">
         <v>325</v>
@@ -4563,25 +4788,25 @@
         <v>307</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="E6" s="17" t="s">
+        <v>308</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>321</v>
+      </c>
+      <c r="G6" s="21" t="s">
         <v>326</v>
-      </c>
-      <c r="F6" s="17" t="s">
-        <v>309</v>
-      </c>
-      <c r="G6" s="17" t="s">
-        <v>327</v>
       </c>
       <c r="H6" s="17" t="s">
         <v>311</v>
       </c>
       <c r="I6" s="17" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>313</v>
+        <v>324</v>
       </c>
       <c r="K6" s="17" t="s">
         <v>75</v>
@@ -4595,8 +4820,8 @@
       <c r="N6" s="17" t="s">
         <v>316</v>
       </c>
-      <c r="O6" s="17" t="s">
-        <v>329</v>
+      <c r="O6" s="17">
+        <v>300</v>
       </c>
       <c r="P6" s="17" t="s">
         <v>74</v>
@@ -4607,34 +4832,34 @@
       <c r="R6" s="17"/>
       <c r="S6" s="17"/>
     </row>
-    <row r="7" spans="1:19" ht="87">
+    <row r="7" spans="1:19" ht="66" customHeight="1">
       <c r="A7" s="19"/>
       <c r="B7" s="17" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C7" s="17" t="s">
         <v>307</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>331</v>
+        <v>308</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>309</v>
-      </c>
-      <c r="G7" s="17" t="s">
-        <v>332</v>
+        <v>329</v>
+      </c>
+      <c r="G7" s="21" t="s">
+        <v>330</v>
       </c>
       <c r="H7" s="17" t="s">
         <v>311</v>
       </c>
       <c r="I7" s="17" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J7" s="17" t="s">
-        <v>313</v>
+        <v>324</v>
       </c>
       <c r="K7" s="17" t="s">
         <v>75</v>
@@ -4648,8 +4873,8 @@
       <c r="N7" s="17" t="s">
         <v>316</v>
       </c>
-      <c r="O7" s="17" t="s">
-        <v>329</v>
+      <c r="O7" s="17">
+        <v>500</v>
       </c>
       <c r="P7" s="17" t="s">
         <v>74</v>
@@ -4660,34 +4885,34 @@
       <c r="R7" s="17"/>
       <c r="S7" s="17"/>
     </row>
-    <row r="8" spans="1:19" ht="72.75">
+    <row r="8" spans="1:19" ht="66" customHeight="1">
       <c r="A8" s="19"/>
       <c r="B8" s="17" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C8" s="17" t="s">
         <v>307</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>335</v>
+        <v>308</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>309</v>
-      </c>
-      <c r="G8" s="17" t="s">
-        <v>336</v>
+        <v>329</v>
+      </c>
+      <c r="G8" s="21" t="s">
+        <v>333</v>
       </c>
       <c r="H8" s="17" t="s">
         <v>311</v>
       </c>
       <c r="I8" s="17" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="J8" s="17" t="s">
-        <v>313</v>
+        <v>324</v>
       </c>
       <c r="K8" s="17" t="s">
         <v>75</v>
@@ -4701,11 +4926,11 @@
       <c r="N8" s="17" t="s">
         <v>316</v>
       </c>
-      <c r="O8" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="P8" s="22">
-        <v>0.06</v>
+      <c r="O8" s="17">
+        <v>500</v>
+      </c>
+      <c r="P8" s="17" t="s">
+        <v>74</v>
       </c>
       <c r="Q8" s="17" t="s">
         <v>74</v>
@@ -4713,10 +4938,10 @@
       <c r="R8" s="17"/>
       <c r="S8" s="17"/>
     </row>
-    <row r="9" spans="1:19" ht="72.75">
+    <row r="9" spans="1:19" ht="66" customHeight="1">
       <c r="A9" s="19"/>
       <c r="B9" s="17" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="C9" s="17" t="s">
         <v>307</v>
@@ -4725,22 +4950,22 @@
         <v>235</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>309</v>
+        <v>329</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="H9" s="17" t="s">
         <v>311</v>
       </c>
       <c r="I9" s="17" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="J9" s="17" t="s">
-        <v>313</v>
+        <v>339</v>
       </c>
       <c r="K9" s="17" t="s">
         <v>75</v>
@@ -4757,8 +4982,8 @@
       <c r="O9" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="P9" s="22">
-        <v>0.06</v>
+      <c r="P9" s="17" t="s">
+        <v>74</v>
       </c>
       <c r="Q9" s="17" t="s">
         <v>74</v>
@@ -4766,10 +4991,10 @@
       <c r="R9" s="17"/>
       <c r="S9" s="17"/>
     </row>
-    <row r="10" spans="1:19" ht="57.75">
+    <row r="10" spans="1:19" ht="66" customHeight="1">
       <c r="A10" s="19"/>
       <c r="B10" s="17" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C10" s="17" t="s">
         <v>307</v>
@@ -4778,19 +5003,19 @@
         <v>235</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>309</v>
+        <v>329</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="H10" s="17" t="s">
         <v>311</v>
       </c>
       <c r="I10" s="17" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="J10" s="17" t="s">
         <v>313</v>
@@ -4810,14 +5035,226 @@
       <c r="O10" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="P10" s="22" t="s">
-        <v>74</v>
-      </c>
-      <c r="Q10" s="17">
-        <v>200</v>
+      <c r="P10" s="17" t="s">
+        <v>344</v>
+      </c>
+      <c r="Q10" s="17" t="s">
+        <v>74</v>
       </c>
       <c r="R10" s="17"/>
       <c r="S10" s="17"/>
+    </row>
+    <row r="11" spans="1:19" ht="66" customHeight="1">
+      <c r="A11" s="19"/>
+      <c r="B11" s="17" t="s">
+        <v>345</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>307</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>235</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>346</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>347</v>
+      </c>
+      <c r="H11" s="17" t="s">
+        <v>311</v>
+      </c>
+      <c r="I11" s="17" t="s">
+        <v>348</v>
+      </c>
+      <c r="J11" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="K11" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="L11" s="17" t="s">
+        <v>314</v>
+      </c>
+      <c r="M11" s="17" t="s">
+        <v>315</v>
+      </c>
+      <c r="N11" s="17" t="s">
+        <v>316</v>
+      </c>
+      <c r="O11" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="P11" s="17" t="s">
+        <v>344</v>
+      </c>
+      <c r="Q11" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="R11" s="17"/>
+      <c r="S11" s="17"/>
+    </row>
+    <row r="12" spans="1:19" ht="66" customHeight="1">
+      <c r="A12" s="19"/>
+      <c r="B12" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>307</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>235</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>350</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>351</v>
+      </c>
+      <c r="H12" s="17" t="s">
+        <v>311</v>
+      </c>
+      <c r="I12" s="17" t="s">
+        <v>352</v>
+      </c>
+      <c r="J12" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="K12" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="L12" s="17" t="s">
+        <v>314</v>
+      </c>
+      <c r="M12" s="17" t="s">
+        <v>315</v>
+      </c>
+      <c r="N12" s="17" t="s">
+        <v>316</v>
+      </c>
+      <c r="O12" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="P12" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q12" s="22">
+        <v>0.06</v>
+      </c>
+      <c r="R12" s="17"/>
+      <c r="S12" s="17"/>
+    </row>
+    <row r="13" spans="1:19" ht="66" customHeight="1">
+      <c r="A13" s="19"/>
+      <c r="B13" s="17" t="s">
+        <v>353</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>307</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>235</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>354</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="G13" s="17" t="s">
+        <v>355</v>
+      </c>
+      <c r="H13" s="17" t="s">
+        <v>311</v>
+      </c>
+      <c r="I13" s="17" t="s">
+        <v>356</v>
+      </c>
+      <c r="J13" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="K13" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="L13" s="17" t="s">
+        <v>314</v>
+      </c>
+      <c r="M13" s="17" t="s">
+        <v>315</v>
+      </c>
+      <c r="N13" s="17" t="s">
+        <v>316</v>
+      </c>
+      <c r="O13" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="P13" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q13" s="22">
+        <v>0.06</v>
+      </c>
+      <c r="R13" s="17"/>
+      <c r="S13" s="17"/>
+    </row>
+    <row r="14" spans="1:19" ht="66" customHeight="1">
+      <c r="A14" s="19"/>
+      <c r="B14" s="17" t="s">
+        <v>357</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>307</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>235</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>358</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="G14" s="17" t="s">
+        <v>359</v>
+      </c>
+      <c r="H14" s="17" t="s">
+        <v>311</v>
+      </c>
+      <c r="I14" s="17" t="s">
+        <v>360</v>
+      </c>
+      <c r="J14" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="K14" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="L14" s="17" t="s">
+        <v>314</v>
+      </c>
+      <c r="M14" s="17" t="s">
+        <v>315</v>
+      </c>
+      <c r="N14" s="17" t="s">
+        <v>316</v>
+      </c>
+      <c r="O14" s="17">
+        <v>200</v>
+      </c>
+      <c r="P14" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q14" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="R14" s="17"/>
+      <c r="S14" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4885,7 +5322,7 @@
         <v>57</v>
       </c>
       <c r="L2" s="23" t="s">
-        <v>346</v>
+        <v>361</v>
       </c>
       <c r="M2" s="23" t="s">
         <v>59</v>
@@ -4908,43 +5345,43 @@
     </row>
     <row r="3" spans="1:18" ht="29.25" customHeight="1">
       <c r="B3" s="25" t="s">
-        <v>347</v>
+        <v>362</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>348</v>
+        <v>363</v>
       </c>
       <c r="D3" s="24" t="s">
         <v>227</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>349</v>
+        <v>364</v>
       </c>
       <c r="F3" s="25" t="s">
-        <v>350</v>
+        <v>365</v>
       </c>
       <c r="G3" s="25" t="s">
-        <v>351</v>
+        <v>366</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
       <c r="I3" s="25" t="s">
-        <v>353</v>
+        <v>368</v>
       </c>
       <c r="J3" s="25" t="s">
-        <v>354</v>
+        <v>369</v>
       </c>
       <c r="K3" s="25" t="s">
-        <v>355</v>
+        <v>370</v>
       </c>
       <c r="L3" s="25" t="s">
-        <v>356</v>
+        <v>371</v>
       </c>
       <c r="M3" s="25" t="s">
-        <v>357</v>
+        <v>372</v>
       </c>
       <c r="N3" s="25" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="O3" s="25" t="s">
         <v>314</v>
@@ -4961,43 +5398,43 @@
     </row>
     <row r="4" spans="1:18" ht="29.25" customHeight="1">
       <c r="B4" s="25" t="s">
-        <v>359</v>
+        <v>374</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>348</v>
+        <v>363</v>
       </c>
       <c r="D4" s="24" t="s">
         <v>235</v>
       </c>
       <c r="E4" s="25" t="s">
-        <v>360</v>
+        <v>375</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>350</v>
+        <v>365</v>
       </c>
       <c r="G4" s="25" t="s">
-        <v>351</v>
+        <v>366</v>
       </c>
       <c r="H4" s="25" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
       <c r="I4" s="25" t="s">
-        <v>361</v>
+        <v>376</v>
       </c>
       <c r="J4" s="25" t="s">
-        <v>362</v>
+        <v>377</v>
       </c>
       <c r="K4" s="25" t="s">
-        <v>363</v>
+        <v>378</v>
       </c>
       <c r="L4" s="25" t="s">
-        <v>364</v>
+        <v>379</v>
       </c>
       <c r="M4" s="25" t="s">
-        <v>357</v>
+        <v>372</v>
       </c>
       <c r="N4" s="25" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="O4" s="25" t="s">
         <v>314</v>
@@ -5014,43 +5451,43 @@
     </row>
     <row r="5" spans="1:18" ht="29.25" customHeight="1">
       <c r="B5" s="25" t="s">
-        <v>365</v>
+        <v>380</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>366</v>
+        <v>381</v>
       </c>
       <c r="D5" s="24" t="s">
         <v>227</v>
       </c>
       <c r="E5" s="25" t="s">
+        <v>382</v>
+      </c>
+      <c r="F5" s="25" t="s">
+        <v>365</v>
+      </c>
+      <c r="G5" s="25" t="s">
+        <v>383</v>
+      </c>
+      <c r="H5" s="25" t="s">
         <v>367</v>
       </c>
-      <c r="F5" s="25" t="s">
-        <v>350</v>
-      </c>
-      <c r="G5" s="25" t="s">
-        <v>368</v>
-      </c>
-      <c r="H5" s="25" t="s">
-        <v>352</v>
-      </c>
       <c r="I5" s="25" t="s">
-        <v>369</v>
+        <v>384</v>
       </c>
       <c r="J5" s="25" t="s">
-        <v>370</v>
+        <v>385</v>
       </c>
       <c r="K5" s="25" t="s">
-        <v>371</v>
+        <v>386</v>
       </c>
       <c r="L5" s="25">
         <v>0</v>
       </c>
       <c r="M5" s="25" t="s">
-        <v>357</v>
+        <v>372</v>
       </c>
       <c r="N5" s="25" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="O5" s="25" t="s">
         <v>314</v>
@@ -5067,43 +5504,43 @@
     </row>
     <row r="6" spans="1:18" ht="28.5" customHeight="1">
       <c r="B6" s="25" t="s">
-        <v>372</v>
+        <v>387</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>366</v>
+        <v>381</v>
       </c>
       <c r="D6" s="24" t="s">
         <v>235</v>
       </c>
       <c r="E6" s="25" t="s">
-        <v>373</v>
+        <v>388</v>
       </c>
       <c r="F6" s="25" t="s">
-        <v>350</v>
+        <v>365</v>
       </c>
       <c r="G6" s="25" t="s">
-        <v>368</v>
+        <v>383</v>
       </c>
       <c r="H6" s="25" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
       <c r="I6" s="25" t="s">
-        <v>374</v>
+        <v>389</v>
       </c>
       <c r="J6" s="25" t="s">
-        <v>375</v>
+        <v>390</v>
       </c>
       <c r="K6" s="25" t="s">
-        <v>376</v>
+        <v>391</v>
       </c>
       <c r="L6" s="25">
         <v>0</v>
       </c>
       <c r="M6" s="25" t="s">
-        <v>357</v>
+        <v>372</v>
       </c>
       <c r="N6" s="25" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="O6" s="25" t="s">
         <v>314</v>
@@ -5120,43 +5557,43 @@
     </row>
     <row r="7" spans="1:18" ht="28.5" customHeight="1">
       <c r="B7" s="25" t="s">
-        <v>377</v>
+        <v>392</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>378</v>
+        <v>393</v>
       </c>
       <c r="D7" s="24" t="s">
         <v>227</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>379</v>
+        <v>394</v>
       </c>
       <c r="F7" s="25" t="s">
-        <v>380</v>
+        <v>395</v>
       </c>
       <c r="G7" s="25" t="s">
-        <v>381</v>
+        <v>396</v>
       </c>
       <c r="H7" s="25" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
       <c r="I7" s="25" t="s">
-        <v>382</v>
+        <v>397</v>
       </c>
       <c r="J7" s="25" t="s">
-        <v>383</v>
+        <v>398</v>
       </c>
       <c r="K7" s="25" t="s">
-        <v>371</v>
+        <v>386</v>
       </c>
       <c r="L7" s="25" t="s">
-        <v>384</v>
+        <v>399</v>
       </c>
       <c r="M7" s="25" t="s">
-        <v>385</v>
+        <v>400</v>
       </c>
       <c r="N7" s="25" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="O7" s="25" t="s">
         <v>314</v>
@@ -5173,43 +5610,43 @@
     </row>
     <row r="8" spans="1:18" ht="28.5" customHeight="1">
       <c r="B8" s="25" t="s">
-        <v>386</v>
+        <v>401</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>378</v>
+        <v>393</v>
       </c>
       <c r="D8" s="24" t="s">
         <v>235</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>387</v>
+        <v>402</v>
       </c>
       <c r="F8" s="25" t="s">
-        <v>380</v>
+        <v>395</v>
       </c>
       <c r="G8" s="25" t="s">
-        <v>381</v>
+        <v>403</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
       <c r="I8" s="25" t="s">
-        <v>388</v>
+        <v>404</v>
       </c>
       <c r="J8" s="25" t="s">
-        <v>389</v>
+        <v>405</v>
       </c>
       <c r="K8" s="25" t="s">
-        <v>376</v>
+        <v>391</v>
       </c>
       <c r="L8" s="25" t="s">
-        <v>390</v>
+        <v>406</v>
       </c>
       <c r="M8" s="25" t="s">
-        <v>385</v>
+        <v>400</v>
       </c>
       <c r="N8" s="25" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="O8" s="25" t="s">
         <v>314</v>
@@ -5226,43 +5663,43 @@
     </row>
     <row r="9" spans="1:18" ht="28.5" customHeight="1">
       <c r="B9" s="25" t="s">
-        <v>391</v>
+        <v>407</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>392</v>
+        <v>408</v>
       </c>
       <c r="D9" s="24" t="s">
         <v>227</v>
       </c>
       <c r="E9" s="25" t="s">
-        <v>393</v>
+        <v>409</v>
       </c>
       <c r="F9" s="25" t="s">
-        <v>380</v>
+        <v>395</v>
       </c>
       <c r="G9" s="25" t="s">
-        <v>394</v>
+        <v>410</v>
       </c>
       <c r="H9" s="25" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
       <c r="I9" s="25" t="s">
-        <v>395</v>
+        <v>411</v>
       </c>
       <c r="J9" s="25" t="s">
-        <v>396</v>
+        <v>412</v>
       </c>
       <c r="K9" s="25" t="s">
-        <v>397</v>
+        <v>413</v>
       </c>
       <c r="L9" s="25">
         <v>0</v>
       </c>
       <c r="M9" s="25" t="s">
-        <v>385</v>
+        <v>400</v>
       </c>
       <c r="N9" s="25" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="O9" s="25" t="s">
         <v>314</v>
@@ -5279,43 +5716,43 @@
     </row>
     <row r="10" spans="1:18" ht="28.5" customHeight="1">
       <c r="B10" s="25" t="s">
-        <v>398</v>
+        <v>414</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>392</v>
+        <v>408</v>
       </c>
       <c r="D10" s="24" t="s">
         <v>235</v>
       </c>
       <c r="E10" s="25" t="s">
-        <v>399</v>
+        <v>415</v>
       </c>
       <c r="F10" s="25" t="s">
-        <v>380</v>
+        <v>395</v>
       </c>
       <c r="G10" s="25" t="s">
-        <v>394</v>
+        <v>410</v>
       </c>
       <c r="H10" s="25" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
       <c r="I10" s="25" t="s">
-        <v>400</v>
+        <v>416</v>
       </c>
       <c r="J10" s="25" t="s">
-        <v>401</v>
+        <v>417</v>
       </c>
       <c r="K10" s="25" t="s">
-        <v>402</v>
+        <v>418</v>
       </c>
       <c r="L10" s="25">
         <v>0</v>
       </c>
       <c r="M10" s="25" t="s">
-        <v>385</v>
+        <v>400</v>
       </c>
       <c r="N10" s="25" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="O10" s="25" t="s">
         <v>314</v>
@@ -5332,43 +5769,43 @@
     </row>
     <row r="11" spans="1:18" ht="28.5" customHeight="1">
       <c r="B11" s="25" t="s">
-        <v>403</v>
+        <v>419</v>
       </c>
       <c r="C11" s="24" t="s">
-        <v>404</v>
+        <v>420</v>
       </c>
       <c r="D11" s="24" t="s">
         <v>227</v>
       </c>
       <c r="E11" s="25" t="s">
-        <v>405</v>
+        <v>421</v>
       </c>
       <c r="F11" s="25" t="s">
-        <v>406</v>
+        <v>422</v>
       </c>
       <c r="G11" s="25" t="s">
-        <v>407</v>
+        <v>423</v>
       </c>
       <c r="H11" s="25" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
       <c r="I11" s="25" t="s">
-        <v>408</v>
+        <v>424</v>
       </c>
       <c r="J11" s="25" t="s">
-        <v>409</v>
+        <v>425</v>
       </c>
       <c r="K11" s="25" t="s">
-        <v>397</v>
+        <v>413</v>
       </c>
       <c r="L11" s="25" t="s">
-        <v>410</v>
+        <v>426</v>
       </c>
       <c r="M11" s="25" t="s">
-        <v>385</v>
+        <v>400</v>
       </c>
       <c r="N11" s="25" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="O11" s="25" t="s">
         <v>314</v>
@@ -5385,43 +5822,43 @@
     </row>
     <row r="12" spans="1:18" ht="28.5" customHeight="1">
       <c r="B12" s="25" t="s">
-        <v>411</v>
+        <v>427</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>404</v>
+        <v>420</v>
       </c>
       <c r="D12" s="24" t="s">
         <v>235</v>
       </c>
       <c r="E12" s="25" t="s">
-        <v>412</v>
+        <v>428</v>
       </c>
       <c r="F12" s="25" t="s">
-        <v>406</v>
+        <v>422</v>
       </c>
       <c r="G12" s="25" t="s">
-        <v>407</v>
+        <v>423</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
       <c r="I12" s="25" t="s">
-        <v>413</v>
+        <v>429</v>
       </c>
       <c r="J12" s="25" t="s">
-        <v>414</v>
+        <v>430</v>
       </c>
       <c r="K12" s="25" t="s">
-        <v>402</v>
+        <v>418</v>
       </c>
       <c r="L12" s="25" t="s">
-        <v>410</v>
+        <v>426</v>
       </c>
       <c r="M12" s="25" t="s">
-        <v>385</v>
+        <v>400</v>
       </c>
       <c r="N12" s="25" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="O12" s="25" t="s">
         <v>314</v>
@@ -5438,34 +5875,34 @@
     </row>
     <row r="13" spans="1:18" ht="43.5">
       <c r="B13" s="25" t="s">
-        <v>415</v>
+        <v>431</v>
       </c>
       <c r="C13" s="24" t="s">
-        <v>416</v>
+        <v>432</v>
       </c>
       <c r="D13" s="24" t="s">
         <v>227</v>
       </c>
       <c r="E13" s="25" t="s">
-        <v>417</v>
+        <v>433</v>
       </c>
       <c r="F13" s="25" t="s">
-        <v>418</v>
+        <v>434</v>
       </c>
       <c r="G13" s="25" t="s">
-        <v>419</v>
+        <v>435</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>420</v>
+        <v>436</v>
       </c>
       <c r="I13" s="25" t="s">
-        <v>421</v>
+        <v>437</v>
       </c>
       <c r="J13" s="25" t="s">
-        <v>422</v>
+        <v>438</v>
       </c>
       <c r="K13" s="25" t="s">
-        <v>355</v>
+        <v>370</v>
       </c>
       <c r="L13" s="25" t="s">
         <v>74</v>
@@ -5474,7 +5911,7 @@
         <v>74</v>
       </c>
       <c r="N13" s="25" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="O13" s="25" t="s">
         <v>314</v>
@@ -5491,7 +5928,7 @@
     </row>
     <row r="14" spans="1:18">
       <c r="B14" s="25" t="s">
-        <v>423</v>
+        <v>439</v>
       </c>
       <c r="C14" s="25"/>
       <c r="D14" s="24"/>
@@ -5500,10 +5937,10 @@
       <c r="G14" s="25"/>
       <c r="H14" s="25"/>
       <c r="I14" s="25" t="s">
-        <v>424</v>
+        <v>440</v>
       </c>
       <c r="J14" s="25" t="s">
-        <v>425</v>
+        <v>441</v>
       </c>
       <c r="K14" s="25"/>
       <c r="L14" s="25"/>
@@ -5516,7 +5953,7 @@
     </row>
     <row r="15" spans="1:18">
       <c r="B15" s="25" t="s">
-        <v>426</v>
+        <v>442</v>
       </c>
       <c r="C15" s="25"/>
       <c r="D15" s="24"/>
@@ -5525,10 +5962,10 @@
       <c r="G15" s="25"/>
       <c r="H15" s="25"/>
       <c r="I15" s="25" t="s">
-        <v>427</v>
+        <v>443</v>
       </c>
       <c r="J15" s="25" t="s">
-        <v>428</v>
+        <v>444</v>
       </c>
       <c r="K15" s="25"/>
       <c r="L15" s="25"/>
@@ -5540,6 +5977,7 @@
       <c r="R15" s="25"/>
     </row>
   </sheetData>
+  <autoFilter ref="B2:R2" xr:uid="{2E015AE2-2662-4C42-BEAE-EB5C4FB0BC06}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>